<commit_message>
feat: two more commodity rules — self_duplicate (intra-respondent) & repeated_token spam; 15 rules total; refresh demo, tests, docs, screenshot
</commit_message>
<xml_diff>
--- a/sample_data/demo_survey.xlsx
+++ b/sample_data/demo_survey.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1416" uniqueCount="807">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1421" uniqueCount="806">
   <si>
     <t>respondent_id</t>
   </si>
@@ -1294,22 +1294,22 @@
     <t>性能令人满意，打算长期用，整体满意</t>
   </si>
   <si>
-    <t>包装还算可以，略有犹豫，门店再多些</t>
-  </si>
-  <si>
-    <t>界面超出预期，会保持关注，价格再优惠就好</t>
-  </si>
-  <si>
-    <t>续航很不错，还会再观望，希望多搞活动</t>
-  </si>
-  <si>
-    <t>质量基本达标，推荐给朋友，颜色再多些</t>
-  </si>
-  <si>
-    <t>续航基本达标，会保持关注，期待新品上市</t>
-  </si>
-  <si>
-    <t>售后稳定可靠，已分享给同事，包装可更环保</t>
+    <t>推荐推荐推荐推荐</t>
+  </si>
+  <si>
+    <t>好的好的好的好的</t>
+  </si>
+  <si>
+    <t>可以可以可以可以</t>
+  </si>
+  <si>
+    <t>满意满意满意满意</t>
+  </si>
+  <si>
+    <t>不错不错不错不错</t>
+  </si>
+  <si>
+    <t>值得值得值得值得</t>
   </si>
   <si>
     <t>口味有点惊艳，会保持关注，期待新品上市</t>
@@ -2084,9 +2084,6 @@
   </si>
   <si>
     <t>音质令人满意，会回购，希望多搞活动</t>
-  </si>
-  <si>
-    <t>使用体验中规中矩，略有犹豫，希望多搞活动</t>
   </si>
   <si>
     <t>包装挺好的，会保持关注，继续加油</t>
@@ -8118,6 +8115,9 @@
       <c r="M124" t="s">
         <v>420</v>
       </c>
+      <c r="N124" t="s">
+        <v>420</v>
+      </c>
     </row>
     <row r="125" spans="1:15">
       <c r="A125" t="s">
@@ -8159,6 +8159,9 @@
       <c r="M125" t="s">
         <v>421</v>
       </c>
+      <c r="N125" t="s">
+        <v>421</v>
+      </c>
     </row>
     <row r="126" spans="1:15">
       <c r="A126" t="s">
@@ -8200,6 +8203,9 @@
       <c r="M126" t="s">
         <v>422</v>
       </c>
+      <c r="N126" t="s">
+        <v>422</v>
+      </c>
       <c r="O126">
         <v>3</v>
       </c>
@@ -8244,6 +8250,9 @@
       <c r="M127" t="s">
         <v>423</v>
       </c>
+      <c r="N127" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="128" spans="1:15">
       <c r="A128" t="s">
@@ -8286,7 +8295,7 @@
         <v>424</v>
       </c>
       <c r="N128" t="s">
-        <v>690</v>
+        <v>424</v>
       </c>
       <c r="O128">
         <v>27</v>
@@ -8332,6 +8341,9 @@
       <c r="M129" t="s">
         <v>425</v>
       </c>
+      <c r="N129" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="130" spans="1:15">
       <c r="A130" t="s">
@@ -8415,7 +8427,7 @@
         <v>427</v>
       </c>
       <c r="N131" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="O131">
         <v>14</v>
@@ -8547,7 +8559,7 @@
         <v>430</v>
       </c>
       <c r="N134" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="135" spans="1:15">
@@ -8632,7 +8644,7 @@
         <v>432</v>
       </c>
       <c r="N136" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="137" spans="1:15">
@@ -8676,7 +8688,7 @@
         <v>433</v>
       </c>
       <c r="N137" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="O137">
         <v>5</v>
@@ -8764,7 +8776,7 @@
         <v>435</v>
       </c>
       <c r="N139" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="140" spans="1:15">
@@ -8808,7 +8820,7 @@
         <v>436</v>
       </c>
       <c r="N140" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="O140">
         <v>22</v>
@@ -8855,7 +8867,7 @@
         <v>437</v>
       </c>
       <c r="N141" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="O141">
         <v>6</v>
@@ -8946,7 +8958,7 @@
         <v>439</v>
       </c>
       <c r="N143" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="O143">
         <v>14</v>
@@ -9037,7 +9049,7 @@
         <v>441</v>
       </c>
       <c r="N145" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="O145">
         <v>14</v>
@@ -9169,7 +9181,7 @@
         <v>444</v>
       </c>
       <c r="N148" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="O148">
         <v>2</v>
@@ -9216,7 +9228,7 @@
         <v>445</v>
       </c>
       <c r="N149" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="O149">
         <v>37</v>
@@ -9263,7 +9275,7 @@
         <v>446</v>
       </c>
       <c r="N150" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="151" spans="1:15">
@@ -9307,7 +9319,7 @@
         <v>447</v>
       </c>
       <c r="N151" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="152" spans="1:15">
@@ -9351,7 +9363,7 @@
         <v>448</v>
       </c>
       <c r="N152" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="153" spans="1:15">
@@ -9395,7 +9407,7 @@
         <v>449</v>
       </c>
       <c r="N153" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="O153">
         <v>38</v>
@@ -9442,7 +9454,7 @@
         <v>450</v>
       </c>
       <c r="N154" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="155" spans="1:15">
@@ -9571,7 +9583,7 @@
         <v>453</v>
       </c>
       <c r="N157" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="O157">
         <v>1</v>
@@ -9700,7 +9712,7 @@
         <v>456</v>
       </c>
       <c r="N160" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="161" spans="1:15">
@@ -9744,7 +9756,7 @@
         <v>457</v>
       </c>
       <c r="N161" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="162" spans="1:15">
@@ -9788,7 +9800,7 @@
         <v>458</v>
       </c>
       <c r="N162" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="163" spans="1:15">
@@ -9832,7 +9844,7 @@
         <v>459</v>
       </c>
       <c r="N163" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="164" spans="1:15">
@@ -9961,7 +9973,7 @@
         <v>462</v>
       </c>
       <c r="N166" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="167" spans="1:15">
@@ -10046,7 +10058,7 @@
         <v>464</v>
       </c>
       <c r="N168" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="169" spans="1:15">
@@ -10090,7 +10102,7 @@
         <v>465</v>
       </c>
       <c r="N169" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="O169">
         <v>8</v>
@@ -10181,7 +10193,7 @@
         <v>467</v>
       </c>
       <c r="N171" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="O171">
         <v>25</v>
@@ -10228,7 +10240,7 @@
         <v>468</v>
       </c>
       <c r="N172" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="173" spans="1:15">
@@ -10272,7 +10284,7 @@
         <v>469</v>
       </c>
       <c r="N173" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="174" spans="1:15">
@@ -10316,7 +10328,7 @@
         <v>470</v>
       </c>
       <c r="N174" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="O174">
         <v>31</v>
@@ -10407,7 +10419,7 @@
         <v>472</v>
       </c>
       <c r="N176" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="O176">
         <v>10</v>
@@ -10498,7 +10510,7 @@
         <v>474</v>
       </c>
       <c r="N178" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="179" spans="1:15">
@@ -10542,7 +10554,7 @@
         <v>475</v>
       </c>
       <c r="N179" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="O179">
         <v>5</v>
@@ -10589,7 +10601,7 @@
         <v>476</v>
       </c>
       <c r="N180" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="O180">
         <v>13</v>
@@ -10636,7 +10648,7 @@
         <v>477</v>
       </c>
       <c r="N181" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="182" spans="1:15">
@@ -10721,7 +10733,7 @@
         <v>479</v>
       </c>
       <c r="N183" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="184" spans="1:15">
@@ -10765,7 +10777,7 @@
         <v>480</v>
       </c>
       <c r="N184" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="O184">
         <v>9</v>
@@ -10812,7 +10824,7 @@
         <v>481</v>
       </c>
       <c r="N185" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="186" spans="1:15">
@@ -10856,7 +10868,7 @@
         <v>482</v>
       </c>
       <c r="N186" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="O186">
         <v>4</v>
@@ -10903,7 +10915,7 @@
         <v>483</v>
       </c>
       <c r="N187" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="188" spans="1:15">
@@ -10947,7 +10959,7 @@
         <v>484</v>
       </c>
       <c r="N188" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="189" spans="1:15">
@@ -10991,7 +11003,7 @@
         <v>485</v>
       </c>
       <c r="N189" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="O189">
         <v>26</v>
@@ -11038,7 +11050,7 @@
         <v>486</v>
       </c>
       <c r="N190" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="191" spans="1:15">
@@ -11082,7 +11094,7 @@
         <v>487</v>
       </c>
       <c r="N191" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="192" spans="1:15">
@@ -11126,7 +11138,7 @@
         <v>488</v>
       </c>
       <c r="N192" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="193" spans="1:15">
@@ -11170,7 +11182,7 @@
         <v>489</v>
       </c>
       <c r="N193" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="194" spans="1:15">
@@ -11255,7 +11267,7 @@
         <v>491</v>
       </c>
       <c r="N195" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="196" spans="1:15">
@@ -11387,7 +11399,7 @@
         <v>494</v>
       </c>
       <c r="N198" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="199" spans="1:15">
@@ -11431,7 +11443,7 @@
         <v>495</v>
       </c>
       <c r="N199" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="O199">
         <v>25</v>
@@ -11478,7 +11490,7 @@
         <v>496</v>
       </c>
       <c r="N200" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="201" spans="1:15">
@@ -11522,7 +11534,7 @@
         <v>497</v>
       </c>
       <c r="N201" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="202" spans="1:15">
@@ -11610,7 +11622,7 @@
         <v>499</v>
       </c>
       <c r="N203" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="204" spans="1:15">
@@ -11654,7 +11666,7 @@
         <v>500</v>
       </c>
       <c r="N204" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="205" spans="1:15">
@@ -11780,7 +11792,7 @@
         <v>503</v>
       </c>
       <c r="N207" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="208" spans="1:15">
@@ -11824,7 +11836,7 @@
         <v>504</v>
       </c>
       <c r="N208" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="O208">
         <v>2</v>
@@ -11871,7 +11883,7 @@
         <v>505</v>
       </c>
       <c r="N209" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="O209">
         <v>5</v>
@@ -11918,7 +11930,7 @@
         <v>506</v>
       </c>
       <c r="N210" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="O210">
         <v>6</v>
@@ -11965,7 +11977,7 @@
         <v>507</v>
       </c>
       <c r="N211" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="212" spans="1:15">
@@ -12009,7 +12021,7 @@
         <v>508</v>
       </c>
       <c r="N212" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="213" spans="1:15">
@@ -12053,7 +12065,7 @@
         <v>509</v>
       </c>
       <c r="N213" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="214" spans="1:15">
@@ -12141,7 +12153,7 @@
         <v>511</v>
       </c>
       <c r="N215" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="216" spans="1:15">
@@ -12185,7 +12197,7 @@
         <v>512</v>
       </c>
       <c r="N216" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="217" spans="1:15">
@@ -12229,7 +12241,7 @@
         <v>513</v>
       </c>
       <c r="N217" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="O217">
         <v>16</v>
@@ -12276,7 +12288,7 @@
         <v>514</v>
       </c>
       <c r="N218" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="219" spans="1:15">
@@ -12320,7 +12332,7 @@
         <v>515</v>
       </c>
       <c r="N219" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="O219">
         <v>21</v>
@@ -12367,7 +12379,7 @@
         <v>516</v>
       </c>
       <c r="N220" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="221" spans="1:15">
@@ -12411,7 +12423,7 @@
         <v>517</v>
       </c>
       <c r="N221" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="222" spans="1:15">
@@ -12455,7 +12467,7 @@
         <v>518</v>
       </c>
       <c r="N222" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="223" spans="1:15">
@@ -12499,7 +12511,7 @@
         <v>519</v>
       </c>
       <c r="N223" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="224" spans="1:15">
@@ -12543,7 +12555,7 @@
         <v>520</v>
       </c>
       <c r="N224" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="225" spans="1:15">
@@ -12587,7 +12599,7 @@
         <v>521</v>
       </c>
       <c r="N225" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="226" spans="1:15">
@@ -12631,7 +12643,7 @@
         <v>522</v>
       </c>
       <c r="N226" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="227" spans="1:15">
@@ -12798,7 +12810,7 @@
         <v>526</v>
       </c>
       <c r="N230" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="231" spans="1:15">
@@ -12927,7 +12939,7 @@
         <v>529</v>
       </c>
       <c r="N233" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="234" spans="1:15">
@@ -12971,7 +12983,7 @@
         <v>530</v>
       </c>
       <c r="N234" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="O234">
         <v>3</v>
@@ -13100,7 +13112,7 @@
         <v>533</v>
       </c>
       <c r="N237" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="O237">
         <v>20</v>
@@ -13191,7 +13203,7 @@
         <v>535</v>
       </c>
       <c r="N239" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="O239">
         <v>27</v>
@@ -13279,7 +13291,7 @@
         <v>537</v>
       </c>
       <c r="N241" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="O241">
         <v>3</v>
@@ -13326,7 +13338,7 @@
         <v>538</v>
       </c>
       <c r="N242" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="243" spans="1:15">
@@ -13370,7 +13382,7 @@
         <v>539</v>
       </c>
       <c r="N243" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O243">
         <v>14</v>
@@ -13417,7 +13429,7 @@
         <v>540</v>
       </c>
       <c r="N244" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="O244">
         <v>1</v>
@@ -13508,7 +13520,7 @@
         <v>542</v>
       </c>
       <c r="N246" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="247" spans="1:15">
@@ -13552,7 +13564,7 @@
         <v>543</v>
       </c>
       <c r="N247" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="248" spans="1:15">
@@ -13596,7 +13608,7 @@
         <v>544</v>
       </c>
       <c r="N248" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="249" spans="1:15">
@@ -13640,7 +13652,7 @@
         <v>545</v>
       </c>
       <c r="N249" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="250" spans="1:15">
@@ -13766,7 +13778,7 @@
         <v>548</v>
       </c>
       <c r="N252" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="O252">
         <v>4</v>
@@ -13813,7 +13825,7 @@
         <v>549</v>
       </c>
       <c r="N253" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="O253">
         <v>16</v>
@@ -13904,7 +13916,7 @@
         <v>551</v>
       </c>
       <c r="N255" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="256" spans="1:15">
@@ -13948,7 +13960,7 @@
         <v>552</v>
       </c>
       <c r="N256" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="O256">
         <v>11</v>
@@ -13995,7 +14007,7 @@
         <v>553</v>
       </c>
       <c r="N257" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="O257">
         <v>23</v>
@@ -14083,7 +14095,7 @@
         <v>555</v>
       </c>
       <c r="N259" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O259">
         <v>23</v>
@@ -14256,7 +14268,7 @@
         <v>559</v>
       </c>
       <c r="N263" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="O263">
         <v>7</v>
@@ -14303,7 +14315,7 @@
         <v>560</v>
       </c>
       <c r="N264" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="265" spans="1:15">
@@ -14388,7 +14400,7 @@
         <v>562</v>
       </c>
       <c r="N266" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="267" spans="1:15">
@@ -14432,7 +14444,7 @@
         <v>563</v>
       </c>
       <c r="N267" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="268" spans="1:15">
@@ -14476,7 +14488,7 @@
         <v>564</v>
       </c>
       <c r="N268" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="269" spans="1:15">
@@ -14608,7 +14620,7 @@
         <v>567</v>
       </c>
       <c r="N271" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="O271">
         <v>22</v>
@@ -14655,7 +14667,7 @@
         <v>568</v>
       </c>
       <c r="N272" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="273" spans="1:15">
@@ -14699,7 +14711,7 @@
         <v>569</v>
       </c>
       <c r="N273" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="O273">
         <v>13</v>
@@ -14746,7 +14758,7 @@
         <v>570</v>
       </c>
       <c r="N274" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="275" spans="1:15">
@@ -14834,7 +14846,7 @@
         <v>572</v>
       </c>
       <c r="N276" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="277" spans="1:15">
@@ -14878,7 +14890,7 @@
         <v>573</v>
       </c>
       <c r="N277" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="O277">
         <v>23</v>
@@ -14966,7 +14978,7 @@
         <v>575</v>
       </c>
       <c r="N279" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="280" spans="1:15">
@@ -15051,7 +15063,7 @@
         <v>577</v>
       </c>
       <c r="N281" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="O281">
         <v>2</v>
@@ -15098,7 +15110,7 @@
         <v>578</v>
       </c>
       <c r="N282" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="O282">
         <v>16</v>
@@ -15145,7 +15157,7 @@
         <v>579</v>
       </c>
       <c r="N283" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="284" spans="1:15">
@@ -15189,7 +15201,7 @@
         <v>580</v>
       </c>
       <c r="N284" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="285" spans="1:15">
@@ -15233,7 +15245,7 @@
         <v>581</v>
       </c>
       <c r="N285" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="286" spans="1:15">
@@ -15277,7 +15289,7 @@
         <v>582</v>
       </c>
       <c r="N286" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="287" spans="1:15">
@@ -15362,7 +15374,7 @@
         <v>584</v>
       </c>
       <c r="N288" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="O288">
         <v>18</v>
@@ -15409,7 +15421,7 @@
         <v>585</v>
       </c>
       <c r="N289" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="290" spans="1:15">
@@ -15453,7 +15465,7 @@
         <v>586</v>
       </c>
       <c r="N290" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="O290">
         <v>11</v>
@@ -15544,7 +15556,7 @@
         <v>588</v>
       </c>
       <c r="N292" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="O292">
         <v>5</v>
@@ -15591,7 +15603,7 @@
         <v>589</v>
       </c>
       <c r="N293" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="O293">
         <v>5</v>
@@ -15638,7 +15650,7 @@
         <v>590</v>
       </c>
       <c r="N294" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="O294">
         <v>13</v>
@@ -15685,7 +15697,7 @@
         <v>591</v>
       </c>
       <c r="N295" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="296" spans="1:15">
@@ -15773,7 +15785,7 @@
         <v>593</v>
       </c>
       <c r="N297" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="298" spans="1:15">
@@ -15902,7 +15914,7 @@
         <v>596</v>
       </c>
       <c r="N300" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="O300">
         <v>13</v>

</xml_diff>